<commit_message>
Improve PMS configuration table and fix imported task generation
</commit_message>
<xml_diff>
--- a/docs/imports/biendong-star-2026/BIENDONG_STAR_2026_Cong_viec_bao_tri_10_thiet_bi.xlsx
+++ b/docs/imports/biendong-star-2026/BIENDONG_STAR_2026_Cong_viec_bao_tri_10_thiet_bi.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Huong_dan" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Maintenance'!A1:Z11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Maintenance'!A1:X11</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -418,7 +418,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z11"/>
+  <dimension ref="A1:X11"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -438,14 +438,12 @@
     <col min="16" max="16" width="22.83203125" customWidth="1"/>
     <col min="17" max="17" width="22.83203125" customWidth="1"/>
     <col min="18" max="18" width="22.83203125" customWidth="1"/>
-    <col min="19" max="19" width="22.83203125" customWidth="1"/>
+    <col min="19" max="19" width="48.83203125" customWidth="1"/>
     <col min="20" max="20" width="22.83203125" customWidth="1"/>
-    <col min="21" max="21" width="48.83203125" customWidth="1"/>
+    <col min="21" max="21" width="22.83203125" customWidth="1"/>
     <col min="22" max="22" width="22.83203125" customWidth="1"/>
     <col min="23" max="23" width="22.83203125" customWidth="1"/>
     <col min="24" max="24" width="22.83203125" customWidth="1"/>
-    <col min="25" max="25" width="22.83203125" customWidth="1"/>
-    <col min="26" max="26" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,39 +496,33 @@
         <v>Review</v>
       </c>
       <c r="Q1" t="str">
-        <v>LastExecutedAt</v>
+        <v>OriginalFrequency</v>
       </c>
       <c r="R1" t="str">
-        <v>LastExecutedRunningHours</v>
+        <v>OriginalLastTime</v>
       </c>
       <c r="S1" t="str">
-        <v>OriginalFrequency</v>
+        <v>OriginalDescription</v>
       </c>
       <c r="T1" t="str">
-        <v>OriginalLastTime</v>
+        <v>Plan</v>
       </c>
       <c r="U1" t="str">
-        <v>OriginalDescription</v>
+        <v>SourceSheet</v>
       </c>
       <c r="V1" t="str">
-        <v>Plan</v>
+        <v>SourceSection</v>
       </c>
       <c r="W1" t="str">
-        <v>SourceSheet</v>
+        <v>SourceRow</v>
       </c>
       <c r="X1" t="str">
-        <v>SourceSection</v>
-      </c>
-      <c r="Y1" t="str">
-        <v>SourceRow</v>
-      </c>
-      <c r="Z1" t="str">
         <v>MonthlyMarks</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>BD26-M-R0009</v>
+        <v>BD26-M-R0009-T-MUSMGUPZ-028575D8</v>
       </c>
       <c r="B2" t="str">
         <v>A001</v>
@@ -578,39 +570,33 @@
         <v/>
       </c>
       <c r="Q2" t="str">
-        <v>2025-08-01</v>
-      </c>
-      <c r="R2" t="str">
-        <v/>
+        <v>M 12</v>
+      </c>
+      <c r="R2">
+        <v>45870</v>
       </c>
       <c r="S2" t="str">
-        <v>M 12</v>
-      </c>
-      <c r="T2">
-        <v>45870</v>
+        <v>Overhauling</v>
+      </c>
+      <c r="T2" t="str">
+        <v/>
       </c>
       <c r="U2" t="str">
-        <v>Overhauling</v>
+        <v>May BD.star 2026</v>
       </c>
       <c r="V2" t="str">
-        <v/>
-      </c>
-      <c r="W2" t="str">
-        <v>May BD.star 2026</v>
+        <v>A</v>
+      </c>
+      <c r="W2">
+        <v>9</v>
       </c>
       <c r="X2" t="str">
-        <v>A</v>
-      </c>
-      <c r="Y2">
-        <v>9</v>
-      </c>
-      <c r="Z2" t="str">
         <v>["","","","","","","","","","","",""]</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>BD26-M-R0010</v>
+        <v>BD26-M-R0010-T-MUSMGUPZ-028575D8</v>
       </c>
       <c r="B3" t="str">
         <v>A002</v>
@@ -658,39 +644,33 @@
         <v/>
       </c>
       <c r="Q3" t="str">
-        <v>2025-08-01</v>
-      </c>
-      <c r="R3" t="str">
-        <v/>
+        <v>M 12</v>
+      </c>
+      <c r="R3">
+        <v>45870</v>
       </c>
       <c r="S3" t="str">
-        <v>M 12</v>
-      </c>
-      <c r="T3">
-        <v>45870</v>
+        <v>Overhauling</v>
+      </c>
+      <c r="T3" t="str">
+        <v/>
       </c>
       <c r="U3" t="str">
-        <v>Overhauling</v>
+        <v>May BD.star 2026</v>
       </c>
       <c r="V3" t="str">
-        <v/>
-      </c>
-      <c r="W3" t="str">
-        <v>May BD.star 2026</v>
+        <v>A</v>
+      </c>
+      <c r="W3">
+        <v>10</v>
       </c>
       <c r="X3" t="str">
-        <v>A</v>
-      </c>
-      <c r="Y3">
-        <v>10</v>
-      </c>
-      <c r="Z3" t="str">
         <v>["","","","","","","","","","","",""]</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>BD26-M-R0011</v>
+        <v>BD26-M-R0011-T-MUSMGUPZ-028575D8</v>
       </c>
       <c r="B4" t="str">
         <v>A003</v>
@@ -738,39 +718,33 @@
         <v/>
       </c>
       <c r="Q4" t="str">
-        <v>2025-08-01</v>
-      </c>
-      <c r="R4" t="str">
-        <v/>
+        <v>M 12</v>
+      </c>
+      <c r="R4">
+        <v>45870</v>
       </c>
       <c r="S4" t="str">
-        <v>M 12</v>
-      </c>
-      <c r="T4">
-        <v>45870</v>
+        <v>Overhauling</v>
+      </c>
+      <c r="T4" t="str">
+        <v/>
       </c>
       <c r="U4" t="str">
-        <v>Overhauling</v>
+        <v>May BD.star 2026</v>
       </c>
       <c r="V4" t="str">
-        <v/>
-      </c>
-      <c r="W4" t="str">
-        <v>May BD.star 2026</v>
+        <v>A</v>
+      </c>
+      <c r="W4">
+        <v>11</v>
       </c>
       <c r="X4" t="str">
-        <v>A</v>
-      </c>
-      <c r="Y4">
-        <v>11</v>
-      </c>
-      <c r="Z4" t="str">
         <v>["","","","","","","","","","","",""]</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>BD26-M-R0012</v>
+        <v>BD26-M-R0012-T-MUSMGUPZ-028575D8</v>
       </c>
       <c r="B5" t="str">
         <v>A004</v>
@@ -818,39 +792,33 @@
         <v/>
       </c>
       <c r="Q5" t="str">
-        <v>2025-09-09</v>
-      </c>
-      <c r="R5" t="str">
-        <v/>
+        <v>H8000</v>
+      </c>
+      <c r="R5">
+        <v>45909</v>
       </c>
       <c r="S5" t="str">
-        <v>H8000</v>
-      </c>
-      <c r="T5">
-        <v>45909</v>
+        <v>Re-tightening</v>
+      </c>
+      <c r="T5" t="str">
+        <v/>
       </c>
       <c r="U5" t="str">
-        <v>Re-tightening</v>
+        <v>May BD.star 2026</v>
       </c>
       <c r="V5" t="str">
-        <v/>
-      </c>
-      <c r="W5" t="str">
-        <v>May BD.star 2026</v>
+        <v>A</v>
+      </c>
+      <c r="W5">
+        <v>12</v>
       </c>
       <c r="X5" t="str">
-        <v>A</v>
-      </c>
-      <c r="Y5">
-        <v>12</v>
-      </c>
-      <c r="Z5" t="str">
         <v>["","","","","","","","","","","",""]</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>BD26-M-R0013</v>
+        <v>BD26-M-R0013-T-MUSMGUPZ-028575D8</v>
       </c>
       <c r="B6" t="str">
         <v>A005</v>
@@ -898,39 +866,33 @@
         <v/>
       </c>
       <c r="Q6" t="str">
-        <v>2025-09-09</v>
-      </c>
-      <c r="R6" t="str">
-        <v/>
+        <v>H 16000</v>
+      </c>
+      <c r="R6">
+        <v>45909</v>
       </c>
       <c r="S6" t="str">
-        <v>H 16000</v>
-      </c>
-      <c r="T6">
-        <v>45909</v>
+        <v>Re-tightening</v>
+      </c>
+      <c r="T6" t="str">
+        <v/>
       </c>
       <c r="U6" t="str">
-        <v>Re-tightening</v>
+        <v>May BD.star 2026</v>
       </c>
       <c r="V6" t="str">
-        <v/>
-      </c>
-      <c r="W6" t="str">
-        <v>May BD.star 2026</v>
+        <v>A</v>
+      </c>
+      <c r="W6">
+        <v>13</v>
       </c>
       <c r="X6" t="str">
-        <v>A</v>
-      </c>
-      <c r="Y6">
-        <v>13</v>
-      </c>
-      <c r="Z6" t="str">
         <v>["","`","","","","","","","","","",""]</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>BD26-M-R0014</v>
+        <v>BD26-M-R0014-T-MUSMGUPZ-028575D8</v>
       </c>
       <c r="B7" t="str">
         <v>A006</v>
@@ -978,39 +940,33 @@
         <v/>
       </c>
       <c r="Q7" t="str">
-        <v>2025-09-11</v>
-      </c>
-      <c r="R7" t="str">
-        <v/>
+        <v>Y 03</v>
+      </c>
+      <c r="R7">
+        <v>45911</v>
       </c>
       <c r="S7" t="str">
-        <v>Y 03</v>
-      </c>
-      <c r="T7">
-        <v>45911</v>
+        <v>Retighten if necessary</v>
+      </c>
+      <c r="T7" t="str">
+        <v/>
       </c>
       <c r="U7" t="str">
-        <v>Retighten if necessary</v>
+        <v>May BD.star 2026</v>
       </c>
       <c r="V7" t="str">
-        <v/>
-      </c>
-      <c r="W7" t="str">
-        <v>May BD.star 2026</v>
+        <v>A</v>
+      </c>
+      <c r="W7">
+        <v>14</v>
       </c>
       <c r="X7" t="str">
-        <v>A</v>
-      </c>
-      <c r="Y7">
-        <v>14</v>
-      </c>
-      <c r="Z7" t="str">
         <v>["","","","","","","","","","","",""]</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>BD26-M-R0015</v>
+        <v>BD26-M-R0015-T-MUSMGUPZ-028575D8</v>
       </c>
       <c r="B8" t="str">
         <v>A007</v>
@@ -1058,39 +1014,33 @@
         <v/>
       </c>
       <c r="Q8" t="str">
-        <v>2025-09-11</v>
-      </c>
-      <c r="R8" t="str">
-        <v/>
+        <v>H10000</v>
+      </c>
+      <c r="R8">
+        <v>45911</v>
       </c>
       <c r="S8" t="str">
-        <v>H10000</v>
-      </c>
-      <c r="T8">
-        <v>45911</v>
+        <v>Check &amp; retighten</v>
+      </c>
+      <c r="T8" t="str">
+        <v/>
       </c>
       <c r="U8" t="str">
-        <v>Check &amp; retighten</v>
+        <v>May BD.star 2026</v>
       </c>
       <c r="V8" t="str">
-        <v/>
-      </c>
-      <c r="W8" t="str">
-        <v>May BD.star 2026</v>
+        <v>A</v>
+      </c>
+      <c r="W8">
+        <v>15</v>
       </c>
       <c r="X8" t="str">
-        <v>A</v>
-      </c>
-      <c r="Y8">
-        <v>15</v>
-      </c>
-      <c r="Z8" t="str">
         <v>["","","","","","","","","","","",""]</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>BD26-M-R0025</v>
+        <v>BD26-M-R0025-T-MUSMGUPZ-028575D8</v>
       </c>
       <c r="B9" t="str">
         <v>A018</v>
@@ -1138,39 +1088,33 @@
         <v/>
       </c>
       <c r="Q9" t="str">
-        <v/>
+        <v>As need</v>
       </c>
       <c r="R9" t="str">
-        <v/>
+        <v>Sep.2025</v>
       </c>
       <c r="S9" t="str">
-        <v>As need</v>
+        <v>Check &amp; adjust timing</v>
       </c>
       <c r="T9" t="str">
-        <v>Sep.2025</v>
+        <v/>
       </c>
       <c r="U9" t="str">
-        <v>Check &amp; adjust timing</v>
+        <v>May BD.star 2026</v>
       </c>
       <c r="V9" t="str">
-        <v/>
-      </c>
-      <c r="W9" t="str">
-        <v>May BD.star 2026</v>
+        <v>A</v>
+      </c>
+      <c r="W9">
+        <v>25</v>
       </c>
       <c r="X9" t="str">
-        <v>A</v>
-      </c>
-      <c r="Y9">
-        <v>25</v>
-      </c>
-      <c r="Z9" t="str">
         <v>["","","","","","","","","","","",""]</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>BD26-M-R0098</v>
+        <v>BD26-M-R0098-T-MUSMGUPZ-028575D8</v>
       </c>
       <c r="B10" t="str">
         <v>A091</v>
@@ -1218,39 +1162,33 @@
         <v/>
       </c>
       <c r="Q10" t="str">
-        <v>2025-09-12</v>
-      </c>
-      <c r="R10" t="str">
-        <v/>
+        <v>Dry dock</v>
+      </c>
+      <c r="R10">
+        <v>45912</v>
       </c>
       <c r="S10" t="str">
-        <v>Dry dock</v>
-      </c>
-      <c r="T10">
-        <v>45912</v>
+        <v>Overhaul</v>
+      </c>
+      <c r="T10" t="str">
+        <v/>
       </c>
       <c r="U10" t="str">
-        <v>Overhaul</v>
+        <v>May BD.star 2026</v>
       </c>
       <c r="V10" t="str">
-        <v/>
-      </c>
-      <c r="W10" t="str">
-        <v>May BD.star 2026</v>
+        <v>A</v>
+      </c>
+      <c r="W10">
+        <v>98</v>
       </c>
       <c r="X10" t="str">
-        <v>A</v>
-      </c>
-      <c r="Y10">
-        <v>98</v>
-      </c>
-      <c r="Z10" t="str">
         <v>["","","","","","","","","","","",""]</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>BD26-D-R0128</v>
+        <v>BD26-D-R0128-T-MUSMGUPZ-028575D8</v>
       </c>
       <c r="B11" t="str">
         <v>3.1.5</v>
@@ -1298,47 +1236,41 @@
         <v/>
       </c>
       <c r="Q11" t="str">
-        <v>2025-12-19</v>
-      </c>
-      <c r="R11" t="str">
-        <v/>
+        <v>chuyÕn</v>
+      </c>
+      <c r="R11">
+        <v>46010</v>
       </c>
       <c r="S11" t="str">
-        <v>chuyÕn</v>
-      </c>
-      <c r="T11">
-        <v>46010</v>
+        <v>ktra biÕn d¹ng, c¾t thay thÕ</v>
+      </c>
+      <c r="T11" t="str">
+        <v/>
       </c>
       <c r="U11" t="str">
-        <v>ktra biÕn d¹ng, c¾t thay thÕ</v>
+        <v>BOONG BD STAR 2026</v>
       </c>
       <c r="V11" t="str">
-        <v/>
-      </c>
-      <c r="W11" t="str">
-        <v>BOONG BD STAR 2026</v>
+        <v>III</v>
+      </c>
+      <c r="W11">
+        <v>128</v>
       </c>
       <c r="X11" t="str">
-        <v>III</v>
-      </c>
-      <c r="Y11">
-        <v>128</v>
-      </c>
-      <c r="Z11" t="str">
         <v>["","","","","","","","","","","",""]</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z11"/>
+  <autoFilter ref="A1:X11"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:X11"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1347,27 +1279,37 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Chọn 10 thiết bị từ file đã tách, giữ tất cả công việc có chu kỳ rõ ràng của các thiết bị này. Không tự thêm công việc.</v>
+        <v>Mã ScheduleCode mới cho đợt thử MUSMGUPZ-028575D8; tránh trùng cấu hình đã xóa mềm. WorkCode và AssetCode giữ nguyên.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Có đủ tháng, năm, giờ, lên đà, theo yêu cầu và theo chuyến. Các dòng cần rà soát không nằm trong mẫu này.</v>
+        <v>Không nhập lịch sử thực hiện hoặc hạn tiếp theo. Hệ thống tự tính lịch từ chu kỳ; ngày nguồn chỉ dùng đối chiếu.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Nhập file thiết bị mẫu trước nếu các AssetCode chưa có trên tàu. Nhóm không tính vào số 10 thiết bị.</v>
+        <v>Chọn 10 thiết bị từ file đã tách, giữ tất cả công việc có chu kỳ rõ ràng của các thiết bị này. Không tự thêm công việc.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>Có đủ tháng, năm, giờ, lên đà, theo yêu cầu và theo chuyến. Các dòng cần rà soát không nằm trong mẫu này.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Nhập file thiết bị mẫu trước nếu các AssetCode chưa có trên tàu. Nhóm không tính vào số 10 thiết bị.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
         <v>ScheduleCode là khóa duy nhất; WorkCode giữ mã công việc nguồn. Import cấu hình, không tự sinh công việc đang chờ thực hiện.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>